<commit_message>
docs: actualizar READMEs de todos los proyectos y correcciones UI
- README de cada servicio con descripción de funcionalidad, lenguaje y tecnología
- Quitar campo Estado KYC del resultado de búsqueda de clientes
- Título de pestaña cambiado a "Intranet Banquito"
- Excel de clientes actualizado con datos reales de empresas y cuenta favorita

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BancoBanQuito_Clientes_Cuentas.xlsx
+++ b/BancoBanQuito_Clientes_Cuentas.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,8 +70,13 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B4F00"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +118,11 @@
         <fgColor rgb="00f0fff4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fce8ff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -188,6 +198,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -27019,33 +27038,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>BancoBanQuito — Catálogo de Clientes Corporativos</t>
+          <t>BancoBanQuito — Catálogo de Empresas Corporativas (EMPRESA_PAGOS_MASIVOS)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>50 empresas masivas | 3 cuentas c/u: CTE=Operativa, NOM=Nómina, AHO=Impuestos/Reservas | Saldo: $1,000.00</t>
+          <t>50 empresas masivas | Subtipo: EMPRESA_PAGOS_MASIVOS | ★ = Cuenta Favorita (usada por SFTP) | Saldo inicial: $1,000.00</t>
         </is>
       </c>
     </row>
@@ -27067,37 +27086,37 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
+          <t>Subtipo</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>N° Cuenta Operativa</t>
-        </is>
-      </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>Suc. Operativa</t>
+          <t>★ N° Cuenta Favorita</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>N° Cuenta Nómina</t>
+          <t>Suc. Favorita</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Suc. Nómina</t>
+          <t>Tipo Cuenta Favorita</t>
         </is>
       </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>N° Cuenta Impuestos</t>
+          <t>Otras Cuentas</t>
         </is>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>Suc. Impuestos</t>
+          <t>Saldo Total</t>
         </is>
       </c>
       <c r="K4" s="12" t="inlineStr">
@@ -27117,47 +27136,45 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Inversiones Andinas del Ecuador S.A.</t>
+          <t>Pacifico Soluciones Financieras 001 S.A.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa1@banquito.com</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>0010000601</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>0010000602</t>
-        </is>
-      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>0010000603</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27172,47 +27189,45 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Comercializadora Pichincha Cía. Ltda.</t>
+          <t>Equinoccio Comercializadora 002 S.A.</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa2@banquito.com</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>0020000604</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>0020000902</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>0020000605</t>
-        </is>
-      </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>0020000606</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27227,47 +27242,45 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Grupo Empresarial Pacífico S.A.</t>
+          <t>Pichincha Logistica Empresarial 003 S.A.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa3@banquito.com</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>0030000607</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>0030000608</t>
-        </is>
-      </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>0030000609</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27282,47 +27295,45 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Importadora Continental Cía. Ltda.</t>
+          <t>Amazonas Consultoria Integral 004 S.A.</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa4@banquito.com</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>0040000610</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>0040000954</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>0040000611</t>
-        </is>
-      </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>0040000612</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27337,47 +27348,45 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Distribuciones Sierra Verde S.A.</t>
+          <t>Sierra Tecnologia Aplicada 005 S.A.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa5@banquito.com</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>0050000613</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>0050000614</t>
-        </is>
-      </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>0050000615</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27392,47 +27401,45 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Tecnologías Innovación Ecuador S.A.</t>
+          <t>Condor Gestion Administrativa 006 S.A.</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa6@banquito.com</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>0010000616</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>0010001456</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>0010000617</t>
-        </is>
-      </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>0010000618</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27447,47 +27454,45 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Construcciones Metropolitanas S.A.</t>
+          <t>Galapagos Servicios Industriales 007 S.A.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa7@banquito.com</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>0020000619</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>0020000621</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>0020000620</t>
-        </is>
-      </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>0020000621</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27502,47 +27507,45 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Agroindustrial Cóndor Cía. Ltda.</t>
+          <t>Capital Servicios Corporativos 008 S.A.</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa8@banquito.com</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>0030000622</t>
-        </is>
-      </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>0030001358</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>0030000623</t>
-        </is>
-      </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>0030000624</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27557,47 +27560,45 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Transportes Nacionales Unidos S.A.</t>
+          <t>Libertad Soluciones Financieras 009 S.A.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa9@banquito.com</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>0040000625</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>0040000626</t>
-        </is>
-      </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>0040000627</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27612,47 +27613,45 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Soluciones Corporativas Andes S.A.</t>
+          <t>Andes Comercializadora 010 S.A.</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa10@banquito.com</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>0050000628</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>0050000760</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>0050000629</t>
-        </is>
-      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>0050000630</t>
-        </is>
-      </c>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27667,47 +27666,45 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Industrias Alimenticias del Norte Cía. Ltda.</t>
+          <t>Pacifico Logistica Empresarial 011 S.A.</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa11@banquito.com</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>0010000631</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>0010000632</t>
-        </is>
-      </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>0010000633</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27722,47 +27719,45 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Grupo Logístico Manabí S.A.</t>
+          <t>Equinoccio Consultoria Integral 012 S.A.</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa12@banquito.com</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>0020000634</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>0020001012</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>0020000635</t>
-        </is>
-      </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I16" s="14" t="inlineStr">
-        <is>
-          <t>0020000636</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27777,47 +27772,45 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Servicios Financieros Austral Cía. Ltda.</t>
+          <t>Pichincha Tecnologia Aplicada 013 S.A.</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa13@banquito.com</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>0030000637</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>0030000638</t>
-        </is>
-      </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>0030000639</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27832,47 +27825,45 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Exportadora Amazónica S.A.</t>
+          <t>Amazonas Gestion Administrativa 014 S.A.</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa14@banquito.com</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>0040000640</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>0040001164</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>0040000641</t>
-        </is>
-      </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>0040000642</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27887,47 +27878,45 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Consultora Empresarial Cuenca Cía. Ltda.</t>
+          <t>Sierra Servicios Industriales 015 S.A.</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa15@banquito.com</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>0050000643</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>0050000644</t>
-        </is>
-      </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>0050000645</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27942,47 +27931,45 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Manufactura Especializada Guayas S.A.</t>
+          <t>Condor Servicios Corporativos 016 S.A.</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa16@banquito.com</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>0010000646</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>0010000916</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>0010000647</t>
-        </is>
-      </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>0010000648</t>
-        </is>
-      </c>
-      <c r="J20" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -27997,47 +27984,45 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Telecomunicaciones Nacionales S.A.</t>
+          <t>Galapagos Soluciones Financieras 017 S.A.</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa17@banquito.com</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>0020000649</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>0020000650</t>
-        </is>
-      </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>0020000651</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28052,47 +28037,45 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Inmobiliaria Capital Norte Cía. Ltda.</t>
+          <t>Capital Comercializadora 018 S.A.</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa18@banquito.com</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>0030000652</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>0030001468</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>0030000653</t>
-        </is>
-      </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>0030000654</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28107,47 +28090,45 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Seguridad Integral Ecuatoriana S.A.</t>
+          <t>Libertad Logistica Empresarial 019 S.A.</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa19@banquito.com</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>0040000655</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>0040000656</t>
-        </is>
-      </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>0040000657</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28162,47 +28143,45 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Farmacéutica Andina Cía. Ltda.</t>
+          <t>Andes Consultoria Integral 020 S.A.</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa20@banquito.com</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>0050000658</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>0050000970</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>0050000659</t>
-        </is>
-      </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>0050000660</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28217,47 +28196,45 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Energía Renovable del Ecuador S.A.</t>
+          <t>Pacifico Tecnologia Aplicada 021 S.A.</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa21@banquito.com</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>0010000661</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>0010000662</t>
-        </is>
-      </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>0010000663</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28272,47 +28249,45 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Textiles del Oriente Cía. Ltda.</t>
+          <t>Equinoccio Gestion Administrativa 022 S.A.</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa22@banquito.com</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>0020000664</t>
-        </is>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>0020001222</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>0020000665</t>
-        </is>
-      </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I26" s="14" t="inlineStr">
-        <is>
-          <t>0020000666</t>
-        </is>
-      </c>
-      <c r="J26" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28327,47 +28302,45 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Automotriz Nacional S.A.</t>
+          <t>Pichincha Servicios Industriales 023 S.A.</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa23@banquito.com</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>0030000667</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>0030000668</t>
-        </is>
-      </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>0030000669</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28382,47 +28355,45 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Hotelería y Turismo Galápagos Cía. Ltda.</t>
+          <t>Amazonas Servicios Corporativos 024 S.A.</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa24@banquito.com</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="F28" s="19" t="inlineStr">
         <is>
           <t>0040000670</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>0040000671</t>
-        </is>
-      </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I28" s="14" t="inlineStr">
-        <is>
-          <t>0040000672</t>
-        </is>
-      </c>
-      <c r="J28" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28437,47 +28408,45 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Alimentos Procesados del Sur S.A.</t>
+          <t>Sierra Soluciones Financieras 025 S.A.</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa25@banquito.com</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>0050000673</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>0050000675</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>0050000674</t>
-        </is>
-      </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>0050000675</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28492,47 +28461,45 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Ingeniería Civil y Arquitectura Cía. Ltda.</t>
+          <t>Condor Comercializadora 026 S.A.</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa26@banquito.com</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>0010000676</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>0010001426</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
-        <is>
-          <t>0010000677</t>
-        </is>
-      </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I30" s="14" t="inlineStr">
-        <is>
-          <t>0010000678</t>
-        </is>
-      </c>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28547,47 +28514,45 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Servicios de Salud Integral S.A.</t>
+          <t>Galapagos Logistica Empresarial 027 S.A.</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa27@banquito.com</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="F31" s="19" t="inlineStr">
         <is>
           <t>0020000679</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>0020000680</t>
-        </is>
-      </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>0020000681</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28602,47 +28567,45 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Tecnología Agropecuaria Nacional Cía. Ltda.</t>
+          <t>Capital Consultoria Integral 028 S.A.</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa28@banquito.com</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>0030000682</t>
-        </is>
-      </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>0030000828</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
-        <is>
-          <t>0030000683</t>
-        </is>
-      </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I32" s="14" t="inlineStr">
-        <is>
-          <t>0030000684</t>
-        </is>
-      </c>
-      <c r="J32" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28657,47 +28620,45 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Retail y Comercio Especializado S.A.</t>
+          <t>Libertad Tecnologia Aplicada 029 S.A.</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa29@banquito.com</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="F33" s="19" t="inlineStr">
         <is>
           <t>0040000685</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>0040000686</t>
-        </is>
-      </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>0040000687</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28712,47 +28673,45 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Grupo Empresarial Tungurahua Cía. Ltda.</t>
+          <t>Andes Gestion Administrativa 030 S.A.</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa30@banquito.com</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>0050000688</t>
-        </is>
-      </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>0050001080</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G34" s="14" t="inlineStr">
-        <is>
-          <t>0050000689</t>
-        </is>
-      </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I34" s="14" t="inlineStr">
-        <is>
-          <t>0050000690</t>
-        </is>
-      </c>
-      <c r="J34" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28767,47 +28726,45 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Distribuciones Comerciales Loja S.A.</t>
+          <t>Pacifico Servicios Industriales 031 S.A.</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa31@banquito.com</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="F35" s="19" t="inlineStr">
         <is>
           <t>0010000691</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>0010000692</t>
-        </is>
-      </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>0010000693</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28822,47 +28779,45 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>Petroquímica Ecuatoriana Cía. Ltda.</t>
+          <t>Equinoccio Servicios Corporativos 032 S.A.</t>
         </is>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa32@banquito.com</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>0020000694</t>
-        </is>
-      </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>0020001332</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
-        <is>
-          <t>0020000695</t>
-        </is>
-      </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I36" s="14" t="inlineStr">
-        <is>
-          <t>0020000696</t>
-        </is>
-      </c>
-      <c r="J36" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28877,47 +28832,45 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Ganadería y Producción Agropecuaria S.A.</t>
+          <t>Pichincha Soluciones Financieras 033 S.A.</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa33@banquito.com</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="F37" s="19" t="inlineStr">
         <is>
           <t>0030000697</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>0030000698</t>
-        </is>
-      </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>0030000699</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28932,47 +28885,45 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>Centro Comercial Metropolitano Cía. Ltda.</t>
+          <t>Amazonas Comercializadora 034 S.A.</t>
         </is>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa34@banquito.com</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>0040000700</t>
-        </is>
-      </c>
-      <c r="F38" s="14" t="inlineStr">
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>0040001484</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
-        <is>
-          <t>0040000701</t>
-        </is>
-      </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I38" s="14" t="inlineStr">
-        <is>
-          <t>0040000702</t>
-        </is>
-      </c>
-      <c r="J38" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K38" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -28987,47 +28938,45 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Producción Audiovisual Nacional S.A.</t>
+          <t>Sierra Logistica Empresarial 035 S.A.</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa35@banquito.com</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="F39" s="19" t="inlineStr">
         <is>
           <t>0050000703</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>0050000704</t>
-        </is>
-      </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>0050000705</t>
-        </is>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29042,47 +28991,45 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>Gestión Ambiental Sostenible Cía. Ltda.</t>
+          <t>Condor Consultoria Integral 036 S.A.</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa36@banquito.com</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>0010000706</t>
-        </is>
-      </c>
-      <c r="F40" s="14" t="inlineStr">
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>0010000708</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>0010000707</t>
-        </is>
-      </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I40" s="14" t="inlineStr">
-        <is>
-          <t>0010000708</t>
-        </is>
-      </c>
-      <c r="J40" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29097,47 +29044,45 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Industria Plástica Especializada S.A.</t>
+          <t>Galapagos Tecnologia Aplicada 037 S.A.</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa37@banquito.com</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="F41" s="19" t="inlineStr">
         <is>
           <t>0020000709</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>0020000710</t>
-        </is>
-      </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>0020000711</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29152,47 +29097,45 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>Operaciones Mineras del Norte Cía. Ltda.</t>
+          <t>Capital Gestion Administrativa 038 S.A.</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa38@banquito.com</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
-        <is>
-          <t>0030000712</t>
-        </is>
-      </c>
-      <c r="F42" s="14" t="inlineStr">
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>0030001038</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G42" s="14" t="inlineStr">
-        <is>
-          <t>0030000713</t>
-        </is>
-      </c>
       <c r="H42" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I42" s="14" t="inlineStr">
-        <is>
-          <t>0030000714</t>
-        </is>
-      </c>
-      <c r="J42" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J42" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K42" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29207,47 +29150,45 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Desarrollo Inmobiliario Moderno S.A.</t>
+          <t>Libertad Servicios Industriales 039 S.A.</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa39@banquito.com</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="F43" s="19" t="inlineStr">
         <is>
           <t>0040000715</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>0040000716</t>
-        </is>
-      </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>0040000717</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29262,47 +29203,45 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>Servicios Informáticos Avanzados Cía. Ltda.</t>
+          <t>Andes Servicios Corporativos 040 S.A.</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa40@banquito.com</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
-        <is>
-          <t>0050000718</t>
-        </is>
-      </c>
-      <c r="F44" s="14" t="inlineStr">
+      <c r="F44" s="19" t="inlineStr">
+        <is>
+          <t>0050001290</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
-        <is>
-          <t>0050000719</t>
-        </is>
-      </c>
       <c r="H44" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I44" s="14" t="inlineStr">
-        <is>
-          <t>0050000720</t>
-        </is>
-      </c>
-      <c r="J44" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K44" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29317,47 +29256,45 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Exportaciones Marítimas Ecuatorianas S.A.</t>
+          <t>Pacifico Soluciones Financieras 041 S.A.</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa41@banquito.com</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="F45" s="19" t="inlineStr">
         <is>
           <t>0010000721</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>0010000722</t>
-        </is>
-      </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>0010000723</t>
-        </is>
-      </c>
-      <c r="J45" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29372,47 +29309,45 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>Procesadora de Alimentos Nativos Cía. Ltda.</t>
+          <t>Equinoccio Comercializadora 042 S.A.</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa42@banquito.com</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
-        <is>
-          <t>0020000724</t>
-        </is>
-      </c>
-      <c r="F46" s="14" t="inlineStr">
+      <c r="F46" s="19" t="inlineStr">
+        <is>
+          <t>0020001442</t>
+        </is>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G46" s="14" t="inlineStr">
-        <is>
-          <t>0020000725</t>
-        </is>
-      </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I46" s="14" t="inlineStr">
-        <is>
-          <t>0020000726</t>
-        </is>
-      </c>
-      <c r="J46" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I46" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J46" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K46" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29427,47 +29362,45 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Construcciones Viales Nacionales S.A.</t>
+          <t>Pichincha Logistica Empresarial 043 S.A.</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa43@banquito.com</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="F47" s="19" t="inlineStr">
         <is>
           <t>0030000727</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>0030000728</t>
-        </is>
-      </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>0030000729</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29482,47 +29415,45 @@
       </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
-          <t>Servicios Educativos Superiores Cía. Ltda.</t>
+          <t>Amazonas Consultoria Integral 044 S.A.</t>
         </is>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa44@banquito.com</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
-        <is>
-          <t>0040000730</t>
-        </is>
-      </c>
-      <c r="F48" s="14" t="inlineStr">
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>0040000844</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G48" s="14" t="inlineStr">
-        <is>
-          <t>0040000731</t>
-        </is>
-      </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I48" s="14" t="inlineStr">
-        <is>
-          <t>0040000732</t>
-        </is>
-      </c>
-      <c r="J48" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I48" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J48" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K48" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29537,47 +29468,45 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Distribución Eléctrica Nacional S.A.</t>
+          <t>Sierra Tecnologia Aplicada 045 S.A.</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa45@banquito.com</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="F49" s="19" t="inlineStr">
         <is>
           <t>0050000733</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>0050000734</t>
-        </is>
-      </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>0050000735</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29592,47 +29521,45 @@
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>Laboratorios del Austro Cía. Ltda.</t>
+          <t>Condor Gestion Administrativa 046 S.A.</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa46@banquito.com</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
-        <is>
-          <t>0010000736</t>
-        </is>
-      </c>
-      <c r="F50" s="14" t="inlineStr">
+      <c r="F50" s="19" t="inlineStr">
+        <is>
+          <t>0010001146</t>
+        </is>
+      </c>
+      <c r="G50" s="14" t="inlineStr">
         <is>
           <t>Sucursal Norte</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr">
-        <is>
-          <t>0010000737</t>
-        </is>
-      </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Norte</t>
-        </is>
-      </c>
-      <c r="I50" s="14" t="inlineStr">
-        <is>
-          <t>0010000738</t>
-        </is>
-      </c>
-      <c r="J50" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Norte</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J50" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K50" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29647,47 +29574,45 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Corporación Manufacturera del Pacífico S.A.</t>
+          <t>Galapagos Servicios Industriales 047 S.A.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa47@banquito.com</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="F51" s="19" t="inlineStr">
         <is>
           <t>0020000739</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>Sucursal Sur</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>0020000740</t>
-        </is>
-      </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Sur</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>0020000741</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Sur</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29702,47 +29627,45 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>Recursos Naturales Amazónicos Cía. Ltda.</t>
+          <t>Capital Servicios Corporativos 048 S.A.</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa48@banquito.com</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
-        <is>
-          <t>0030000742</t>
-        </is>
-      </c>
-      <c r="F52" s="14" t="inlineStr">
+      <c r="F52" s="19" t="inlineStr">
+        <is>
+          <t>0030001148</t>
+        </is>
+      </c>
+      <c r="G52" s="14" t="inlineStr">
         <is>
           <t>Sucursal Centro</t>
         </is>
       </c>
-      <c r="G52" s="14" t="inlineStr">
-        <is>
-          <t>0030000743</t>
-        </is>
-      </c>
       <c r="H52" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Centro</t>
-        </is>
-      </c>
-      <c r="I52" s="14" t="inlineStr">
-        <is>
-          <t>0030000744</t>
-        </is>
-      </c>
-      <c r="J52" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Centro</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K52" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29757,47 +29680,45 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Innovación Biotecnológica Ecuador S.A.</t>
+          <t>Libertad Soluciones Financieras 049 S.A.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
           <t>contacto.empresa49@banquito.com</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>0040000745</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>0040000747</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>Sucursal Valles</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>0040000746</t>
-        </is>
-      </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>Sucursal Valles</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>0040000747</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr">
-        <is>
-          <t>Sucursal Valles</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
@@ -29812,223 +29733,160 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>Servicios Portuarios Nacionales Cía. Ltda.</t>
+          <t>Andes Comercializadora 050 S.A.</t>
         </is>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
           <t>contacto.empresa50@banquito.com</t>
         </is>
       </c>
-      <c r="E54" s="14" t="inlineStr">
-        <is>
-          <t>0050000748</t>
-        </is>
-      </c>
-      <c r="F54" s="14" t="inlineStr">
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>0050001400</t>
+        </is>
+      </c>
+      <c r="G54" s="14" t="inlineStr">
         <is>
           <t>Sucursal Digital</t>
         </is>
       </c>
-      <c r="G54" s="14" t="inlineStr">
-        <is>
-          <t>0050000749</t>
-        </is>
-      </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>Sucursal Digital</t>
-        </is>
-      </c>
-      <c r="I54" s="14" t="inlineStr">
-        <is>
-          <t>0050000750</t>
-        </is>
-      </c>
-      <c r="J54" s="14" t="inlineStr">
-        <is>
-          <t>Sucursal Digital</t>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>$18,000.00</t>
         </is>
       </c>
       <c r="K54" s="14" t="inlineStr">
         <is>
-          <t>Pagos Masivos</t>
+          <t>Acceso SFTP</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>── Empresas Demo (sin cuentas automáticas) ──</t>
+          <t>── Empresas Demo (subtype EMPRESA_PAGOS_MASIVOS, cuentas creadas via API) ──</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="B56" s="10" t="inlineStr">
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>1753451481001</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>Venta de Autos</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="inlineStr">
+        <is>
+          <t>estefylove09@gmail.com</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>0016618965</t>
+        </is>
+      </c>
+      <c r="G56" s="21" t="inlineStr">
+        <is>
+          <t>Sucursal Norte</t>
+        </is>
+      </c>
+      <c r="H56" s="21" t="inlineStr">
+        <is>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I56" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="20" t="inlineStr">
+        <is>
+          <t>$1,000.00</t>
+        </is>
+      </c>
+      <c r="K56" s="21" t="inlineStr">
+        <is>
+          <t>★ Demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="inlineStr">
         <is>
           <t>1757158215001</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
+      <c r="C57" s="21" t="inlineStr">
         <is>
           <t>TechSolutions Ecuador S.A.</t>
         </is>
       </c>
-      <c r="D56" s="10" t="inlineStr">
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>EMPRESA_PAGOS_MASIVOS</t>
+        </is>
+      </c>
+      <c r="E57" s="21" t="inlineStr">
         <is>
           <t>info@techsolutions.ec</t>
         </is>
       </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J56" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K56" s="10" t="inlineStr">
-        <is>
-          <t>★ Demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>1791234567001</t>
-        </is>
-      </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>Importadora Andina Cía. Ltda.</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>contacto@importandina.ec</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J57" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K57" s="10" t="inlineStr">
-        <is>
-          <t>★ Demo</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>1791765432001</t>
-        </is>
-      </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>Distribuidora El Comercio S.A.</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>gerencia@distcomercio.ec</t>
-        </is>
-      </c>
-      <c r="E58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J58" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K58" s="10" t="inlineStr">
+      <c r="F57" s="19" t="inlineStr">
+        <is>
+          <t>0047600277</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="inlineStr">
+        <is>
+          <t>Sucursal Valles</t>
+        </is>
+      </c>
+      <c r="H57" s="21" t="inlineStr">
+        <is>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="I57" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="20" t="inlineStr">
+        <is>
+          <t>$1,000.00</t>
+        </is>
+      </c>
+      <c r="K57" s="21" t="inlineStr">
         <is>
           <t>★ Demo</t>
         </is>

</xml_diff>